<commit_message>
Add new Excel templates for P2 project, including P2_Form_BP_Cong_Nghe and individual member files. Implement scripts for generating evaluations, inspecting forms, and applying mapping rules. Update formulas and add meeting notes for 02-02-2026.
</commit_message>
<xml_diff>
--- a/P2_Form_BP_Cong_Nghe.xlsx
+++ b/P2_Form_BP_Cong_Nghe.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CONG VIEC\project-management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E9FB08-1BE3-42F5-AB74-823DDD145D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419EF955-328D-4588-8401-32568C023203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Cấu trúc &amp; Trọng số" sheetId="2" r:id="rId2"/>
-    <sheet name="Product_Engineer" sheetId="4" r:id="rId3"/>
-    <sheet name="MÔ TẢ - PHỤ LỤC" sheetId="5" r:id="rId4"/>
-    <sheet name="Summary_Ranking" sheetId="3" state="hidden" r:id="rId5"/>
+    <sheet name="Product_Engineer" sheetId="3" r:id="rId3"/>
+    <sheet name="MÔ TẢ - PHỤ LỤC" sheetId="4" r:id="rId4"/>
+    <sheet name="Summary_Ranking" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,9 +37,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="151">
   <si>
     <t>P2+ - MÔ HÌNH ĐÁNH GIÁ NĂNG LỰC MỞ RỘNG</t>
+  </si>
+  <si>
+    <t>P2+ là mô hình đánh giá năng lực mở rộng, trong đó kết quả thực hiện OKR/KPI được tích hợp như một thành phần của P2, thay vì tách thành P3 độc lập. Mục tiêu là đơn giản hóa quy trình, phản ánh đúng đặc thù công việc kỹ thuật và đảm bảo đánh giá cân bằng giữa năng lực dài hạn và kết quả ngắn hạn.</t>
   </si>
   <si>
     <t>👉 Lưu ý quan trọng:</t>
@@ -53,13 +56,13 @@
     <t>CẤU TRÚC &amp; TRỌNG SỐ P2+</t>
   </si>
   <si>
-    <t>1️⃣ CẤU TRÚC TỔNG THỂ P2+</t>
+    <t>I. CẤU TRÚC TỔNG THỂ P2+</t>
   </si>
   <si>
     <t>P2+ gồm 2 thành phần:</t>
   </si>
   <si>
-    <t>A. P2-Core – Năng lực &amp; cách làm việc (70%)</t>
+    <t>A. P2-Core – Năng lực &amp; cách làm việc (50%)</t>
   </si>
   <si>
     <t xml:space="preserve">  • A. Năng lực kỹ thuật</t>
@@ -74,7 +77,7 @@
     <t xml:space="preserve">  • D. AI Agent &amp; Cải tiến</t>
   </si>
   <si>
-    <t>B. P2-Delivery – Kết quả công việc (30%)</t>
+    <t>B. P2-Delivery – Kết quả công việc (50%)</t>
   </si>
   <si>
     <t xml:space="preserve">  • OKR/KPI tháng hoặc quý</t>
@@ -83,13 +86,13 @@
     <t xml:space="preserve">  • Chất lượng delivery</t>
   </si>
   <si>
-    <t>III. CÁCH TÍNH ĐIỂM P2+</t>
+    <t>II. CÁCH TÍNH ĐIỂM P2+</t>
   </si>
   <si>
     <t>P2+ là điểm đánh giá cuối cùng dùng để xếp loại năng lực.</t>
   </si>
   <si>
-    <t>P2+ Tổng = (P2-Core × 70%) + (P2-Delivery × 30%)</t>
+    <t>P2+ Tổng = (P2-Core × 50%) + (P2-Delivery × 50%)</t>
   </si>
   <si>
     <t>📌 Trong đó:</t>
@@ -101,7 +104,7 @@
     <t>P2-Delivery: phản ánh kết quả thực tế trong kỳ</t>
   </si>
   <si>
-    <t>IV. NGUYÊN TẮC ĐÁNH GIÁ (BẮT BUỘC TUÂN THỦ)</t>
+    <t>III. NGUYÊN TẮC ĐÁNH GIÁ (BẮT BUỘC TUÂN THỦ)</t>
   </si>
   <si>
     <t>1️⃣ Không chấm trùng nội dung</t>
@@ -131,7 +134,7 @@
     <t xml:space="preserve">  • Không đánh giá theo 1–2 tình huống nổi bật</t>
   </si>
   <si>
-    <t>V. NGƯỠNG XẾP LOẠI</t>
+    <t>IV. NGƯỠNG XẾP LOẠI</t>
   </si>
   <si>
     <t>P2+ Tổng</t>
@@ -164,6 +167,291 @@
     <t>Xuất sắc</t>
   </si>
   <si>
+    <t>P2 PERFORMANCE EVALUATION – Product Engineer</t>
+  </si>
+  <si>
+    <t>Họ và tên</t>
+  </si>
+  <si>
+    <t>Kỳ đánh giá</t>
+  </si>
+  <si>
+    <t>Vai trò</t>
+  </si>
+  <si>
+    <t>Người đánh giá</t>
+  </si>
+  <si>
+    <t>Nhóm năng lực</t>
+  </si>
+  <si>
+    <t>Trọng số (%)</t>
+  </si>
+  <si>
+    <t>Mức (L1/L2/L3)</t>
+  </si>
+  <si>
+    <t>Điểm quy đổi</t>
+  </si>
+  <si>
+    <t>Nhận xét</t>
+  </si>
+  <si>
+    <t>A. Năng lực kỹ thuật</t>
+  </si>
+  <si>
+    <t>B. Ownership &amp; trách nhiệm</t>
+  </si>
+  <si>
+    <t>C. DevOps &amp; vận hành (bắt buộc)</t>
+  </si>
+  <si>
+    <t>D. AI Agent &amp; cải tiến (bắt buộc)</t>
+  </si>
+  <si>
+    <t>TỔNG P2</t>
+  </si>
+  <si>
+    <t>THANG ĐÁNH GIÁ CHI TIẾT (L1/L2/L3)</t>
+  </si>
+  <si>
+    <t>Mức</t>
+  </si>
+  <si>
+    <t>Mô tả</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>Thực hiện được các phần việc rõ ràng khi có hướng dẫn; cần review thường xuyên; chất lượng chưa ổn định.</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>Tự triển khai độc lập; chất lượng ổn định, ít rework; chủ động xử lý rủi ro và cải thiện sản phẩm.</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>Extra: Không chỉ hoàn thành tốt phần việc cá nhân mà còn cải tiến hệ thống, chuẩn hoá cách làm và lan toả kinh nghiệm cho nhóm.</t>
+  </si>
+  <si>
+    <t>Kết quả công việc (P2-Delivery – từ OKR/KPI)</t>
+  </si>
+  <si>
+    <t>Phần này phản ánh kết quả đầu ra, không đánh giá lại năng lực hay cách làm việc. (P2-Core là phần đánh giá NĂNG LỰC &amp; CÁCH LÀM VIỆC mang tính nền tảng và dài hạn của nhân sự Công Nghệ.)</t>
+  </si>
+  <si>
+    <t>Tiêu chí</t>
+  </si>
+  <si>
+    <t>Điểm (Chưa đạt=1.5, Đạt=3.5, Tốt=5)</t>
+  </si>
+  <si>
+    <t>Mức độ hoàn thành OKR</t>
+  </si>
+  <si>
+    <t>Tỷ lệ hoàn thành các mục tiêu đã cam kết trong kỳ đánh giá</t>
+  </si>
+  <si>
+    <t>Chất lượng kết quả</t>
+  </si>
+  <si>
+    <t>Ít lỗi nghiêm trọng; hạn chế làm lại; không gây rủi ro hệ thống</t>
+  </si>
+  <si>
+    <t>Cam kết &amp; tiến độ</t>
+  </si>
+  <si>
+    <t>Hoàn thành đúng hạn; chủ động báo sớm rủi ro; phối hợp tốt</t>
+  </si>
+  <si>
+    <t>P2-Delivery = Trung bình cộng các tiêu chí trên</t>
+  </si>
+  <si>
+    <t>P2-Delivery</t>
+  </si>
+  <si>
+    <t>MÔ TẢ NĂNG LỰC THEO VAI TRÒ</t>
+  </si>
+  <si>
+    <t>Gợi ý: dùng nút +/- (Outline) để thu gọn/mở rộng theo từng Vai trò. Cấp độ 1 (Thực thi – phối hợp): Làm tốt phần việc kỹ thuật của mình | Cấp độ 2 (Chủ động – cải tiến): Giải quyết bài toán xuyên hệ thống | Cấp độ 3 (Chuẩn hoá – dẫn dắt): Định hướng, tạo chuẩn, mở rộng</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>Cấp độ 1</t>
+  </si>
+  <si>
+    <t>Cấp độ 2</t>
+  </si>
+  <si>
+    <t>Cấp độ 3</t>
+  </si>
+  <si>
+    <t>Tự triển khai tính năng (API + DB); code dễ đọc; tests cơ bản; xử lý trường hợp lỗi không mong muốn xảy ra.</t>
+  </si>
+  <si>
+    <t>Thiết kế kiến trúc/module gọn; cải thiện performance/security; tests chắc; nâng chất lượng qua review.</t>
+  </si>
+  <si>
+    <t>Định hướng kiến trúc hệ thống có khả năng mở rộng; chủ động ngăn ngừa rủi ro và lỗi hệ thống; dẫn dắt cải tiến kỹ thuật lớn và hỗ trợ nâng cao năng lực đội ngũ.</t>
+  </si>
+  <si>
+    <t>Bàn giao công việc ổn định; biết tách công việc thành các đầu việc rõ ràng; chịu trách nhiệm xử lý lỗi đến khi hoàn tất; chủ động báo sớm các rủi ro phát sinh.</t>
+  </si>
+  <si>
+    <t>Chủ động quản lý phạm vi và rủi ro công việc; phối hợp hiệu quả với các bộ phận liên quan; giảm phát sinh làm lại nhờ yêu cầu và tài liệu được chuẩn bị rõ ràng.</t>
+  </si>
+  <si>
+    <t>Cải tiến quy trình bàn giao công việc trong đội (tiêu chí hoàn thành, danh sách rà soát); xử lý các điểm nghẽn trong phối hợp giữa các nhóm; nâng cao khả năng dự báo và kiểm soát tiến độ chung.</t>
+  </si>
+  <si>
+    <t>C. DevOps &amp; vận hành</t>
+  </si>
+  <si>
+    <t>Thực hiện quy trình tích hợp và triển khai tự động; hiểu và sử dụng đúng cấu hình môi trường, thông tin bảo mật; theo dõi nhật ký và lỗi hệ thống; tham gia trực xử lý sự cố khi cần.</t>
+  </si>
+  <si>
+    <t>Chủ động cải thiện quy trình triển khai (tối ưu hiệu năng, kiểm soát chất lượng); bổ sung theo dõi chỉ số và cảnh báo; thực hiện phương án quay lui khi có sự cố; nâng cao độ ổn định và rút ngắn thời gian khắc phục lỗi.</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa quy trình phát hành và giám sát hệ thống; xây dựng hướng dẫn vận hành và xử lý sự cố; chủ trì phân tích nguyên nhân sau sự cố; hướng dẫn và nâng cao năng lực vận hành cho đội ngũ.</t>
+  </si>
+  <si>
+    <t>D. AI Agent &amp; cải tiến</t>
+  </si>
+  <si>
+    <t>Sử dụng AI Agent để hỗ trợ code, chỉnh sửa code, viết kiểm thử và tìm lỗi; biết đặt yêu cầu rõ ràng; luôn kiểm tra lại kết quả trước khi áp dụng.</t>
+  </si>
+  <si>
+    <t>Xây dựng mẫu yêu cầu và quy trình làm việc có thể tái sử dụng; dùng AI để hỗ trợ rà soát và tìm lỗi; theo dõi hiệu quả bằng các chỉ số như thời gian hoàn thành và tỷ lệ lỗi phát sinh.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong kỹ thuật một cách có kiểm soát; đào tạo và hướng dẫn đội ngũ; tự động hóa các công việc lặp lại theo nguyên tắc an toàn, phân quyền và tuân thủ quy định nội bộ.</t>
+  </si>
+  <si>
+    <t>Designer</t>
+  </si>
+  <si>
+    <t>Tự xây dựng luồng trải nghiệm và đặc tả giao diện; đảm bảo tính nhất quán về hình ảnh; bàn giao thiết kế rõ ràng để đội triển khai chính xác.</t>
+  </si>
+  <si>
+    <t>Cải thiện khả năng sử dụng dựa trên nghiên cứu và đánh giá trải nghiệm; phát triển và mở rộng hệ thống thiết kế; giảm phát sinh làm lại nhờ đặc tả thiết kế rõ ràng.</t>
+  </si>
+  <si>
+    <t>Định hướng thiết kế tổng thể; tạo ra tác động trải nghiệm người dùng có thể đo lường; quản trị và chuẩn hóa hệ thống thiết kế; hướng dẫn và kết nối các đội cùng áp dụng.</t>
+  </si>
+  <si>
+    <t>Bàn giao công việc ổn định; xác định rõ phạm vi; lặp lại thiết kế kịp thời; phối hợp sớm với các bên triển khai để thống nhất ràng buộc.</t>
+  </si>
+  <si>
+    <t>Quản lý các lựa chọn và đánh đổi trong thiết kế; chuẩn bị phương án thay thế; ghi nhận rõ các quyết định; giảm phát sinh làm lại thông qua rà soát thiết kế.</t>
+  </si>
+  <si>
+    <t>Nâng chuẩn bàn giao thiết kế (tiêu chí hoàn thành, danh sách rà soát); tháo gỡ các vướng mắc phối hợp giữa các đội; nâng cao khả năng dự báo và kiểm soát tiến độ.</t>
+  </si>
+  <si>
+    <t>Làm việc với môi trường preview và staging; sử dụng nhất quán các thành phần và chuẩn thiết kế; xây dựng đặc tả phù hợp với khả năng triển khai.</t>
+  </si>
+  <si>
+    <t>Thúc đẩy áp dụng chuẩn thành phần thiết kế; cải thiện tự động hóa bàn giao thiết kế–triển khai; giảm lỗi tích hợp và công việc làm lại.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt chuẩn hóa quy trình thiết kế–triển khai với đội phát triển; xây dựng hướng dẫn và các thực hành tốt cho toàn đội.</t>
+  </si>
+  <si>
+    <t>Sử dụng AI để hỗ trợ xây dựng khung thiết kế, nội dung trải nghiệm và phương án thiết kế; biết đặt yêu cầu phù hợp; kiểm tra và đối chiếu với hệ thống thiết kế hiện có.</t>
+  </si>
+  <si>
+    <t>Xây dựng thư viện yêu cầu AI có thể tái sử dụng; tăng tốc tổng hợp nghiên cứu; theo dõi tác động của AI đến thời gian thực hiện và mức độ làm lại.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong thiết kế một cách an toàn và có kiểm soát; đào tạo đội ngũ; tự động hóa các công việc lặp lại theo quy định và chuẩn quản trị.</t>
+  </si>
+  <si>
+    <t>FrontEnd</t>
+  </si>
+  <si>
+    <t>Tự triển khai tính năng giao diện từ đầu đến cuối (giao diện, trạng thái, tích hợp dữ liệu); xử lý các tình huống phát sinh; viết mã rõ ràng, dễ bảo trì.</t>
+  </si>
+  <si>
+    <t>Cải thiện hiệu năng và khả năng truy cập của giao diện; xây dựng thành phần dùng lại; nâng cao kiến trúc và kiểm thử để tăng độ ổn định.</t>
+  </si>
+  <si>
+    <t>Định hướng kỹ thuật frontend; dẫn dắt các thay đổi lớn để giảm rủi ro; hướng dẫn đội ngũ; chủ động ngăn ngừa lỗi ảnh hưởng diện rộng trên giao diện.</t>
+  </si>
+  <si>
+    <t>Bàn giao công việc ổn định; chịu trách nhiệm xử lý lỗi đến khi hoàn tất; phối hợp sớm với backend và thiết kế; chủ động báo rủi ro.</t>
+  </si>
+  <si>
+    <t>Quản lý các lựa chọn và đánh đổi về trải nghiệm người dùng; giảm phát sinh làm lại; nâng chất lượng bàn giao bằng đặc tả, minh chứng và tài liệu rõ ràng.</t>
+  </si>
+  <si>
+    <t>Nâng chuẩn bàn giao và rà soát (chuẩn thành phần, danh sách rà soát); tháo gỡ vướng mắc phối hợp giữa các đội; nâng cao khả năng dự báo và kiểm soát tiến độ.</t>
+  </si>
+  <si>
+    <t>Sử dụng thành thạo quy trình tích hợp và triển khai; quản lý cấu hình môi trường; theo dõi lỗi phía người dùng; giữ bản phát hành gọn và ổn định.</t>
+  </si>
+  <si>
+    <t>Cải thiện quy trình triển khai (tối ưu tốc độ, kiểm soát chất lượng); giảm kích thước và thời gian tải; có phương án quay lui khi sự cố; nâng cao độ ổn định.</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa phát hành và giám sát cho frontend; xây dựng hướng dẫn xử lý sự cố; hướng dẫn đội ngũ thực hành vận hành; giảm lỗi phía người dùng và rút ngắn thời gian khắc phục.</t>
+  </si>
+  <si>
+    <t>Sử dụng AI để hỗ trợ tạo khung code, chỉnh sửa code, viết kiểm thử và tìm lỗi; biết đặt yêu cầu rõ ràng; luôn kiểm tra lại trước khi áp dụng.</t>
+  </si>
+  <si>
+    <t>Xây dựng mẫu yêu cầu AI có thể tái sử dụng (thành phần, khả năng truy cập, kiểm thử); dùng AI hỗ trợ rà soát và cải tiến mã; theo dõi hiệu quả bằng các chỉ số phù hợp.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong frontend theo quy chuẩn; đào tạo đội ngũ; tự động hóa các công việc lặp lại một cách an toàn và có kiểm soát.</t>
+  </si>
+  <si>
+    <t>FullStack</t>
+  </si>
+  <si>
+    <t>Tự triển khai tính năng từ đầu đến cuối (giao diện, xử lý dữ liệu, lưu trữ); đảm bảo chất lượng cơ bản; viết kiểm thử cần thiết; xử lý các tình huống lỗi phát sinh.</t>
+  </si>
+  <si>
+    <t>Phân định rõ trách nhiệm giữa backend và frontend; cải thiện hiệu năng và an toàn hệ thống; thực hiện tái cấu trúc có kiểm soát; xây dựng kiểm thử vững chắc hơn.</t>
+  </si>
+  <si>
+    <t>Định hướng kỹ thuật end-to-end; chủ động ngăn ngừa rủi ro và lỗi hệ thống; hướng dẫn đội ngũ; dẫn dắt các đợt tái cấu trúc và chuyển đổi hệ thống lớn một cách an toàn.</t>
+  </si>
+  <si>
+    <t>Chịu trách nhiệm toàn bộ tính năng từ đầu đến cuối; đảm bảo vận hành ổn định; chủ động báo rủi ro; xử lý triệt để vấn đề đến khi hoàn tất.</t>
+  </si>
+  <si>
+    <t>Quản lý phạm vi và rủi ro công việc; trao đổi và thống nhất các đánh đổi kỹ thuật; giảm phát sinh làm lại; cải thiện chất lượng tài liệu và bàn giao.</t>
+  </si>
+  <si>
+    <t>Nâng cao khả năng dự báo; xây dựng và áp dụng các chuẩn chung (tiêu chí hoàn thành, danh sách rà soát); tháo gỡ vướng mắc trong phối hợp giữa các đội.</t>
+  </si>
+  <si>
+    <t>Sử dụng quy trình tích hợp và triển khai tự động; quản lý cấu hình và thông tin bảo mật; theo dõi lỗi và nhật ký hệ thống; triển khai an toàn và tham gia trực xử lý sự cố.</t>
+  </si>
+  <si>
+    <t>Cải thiện quy trình triển khai; bổ sung theo dõi chỉ số và cảnh báo; có phương án quay lui khi cần; nâng cao độ ổn định trên toàn bộ hệ thống.</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa phát hành và giám sát hệ thống; xây dựng hướng dẫn vận hành và xử lý sự cố; giảm thời gian khắc phục lỗi; hướng dẫn đội ngũ thực hành vận hành hiệu quả.</t>
+  </si>
+  <si>
+    <t>Sử dụng AI hỗ trợ toàn bộ chuỗi phát triển (tạo khung, chỉnh sửa code, kiểm thử, tìm lỗi); biết đặt yêu cầu phù hợp; luôn rà soát kỹ kết quả trước khi áp dụng.</t>
+  </si>
+  <si>
+    <t>Xây dựng mẫu yêu cầu và quy trình làm việc với AI có thể tái sử dụng; dùng AI hỗ trợ rà soát và tìm lỗi; theo dõi tác động đến thời gian thực hiện và chất lượng.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong phát triển end-to-end một cách an toàn và có kiểm soát; đào tạo đội ngũ; tự động hóa các công việc xuyên suốt theo chuẩn quản trị.</t>
+  </si>
+  <si>
     <t>P2 SUMMARY &amp; RANKING – BP CÔNG NGHỆ</t>
   </si>
   <si>
@@ -173,15 +461,6 @@
     <t>STT</t>
   </si>
   <si>
-    <t>Họ và tên</t>
-  </si>
-  <si>
-    <t>Vai trò</t>
-  </si>
-  <si>
-    <t>Kỳ đánh giá</t>
-  </si>
-  <si>
     <t>Điểm P2</t>
   </si>
   <si>
@@ -213,289 +492,13 @@
   </si>
   <si>
     <t>Nguyễn Đăng Đức</t>
-  </si>
-  <si>
-    <t>P2 PERFORMANCE EVALUATION – Product Engineer</t>
-  </si>
-  <si>
-    <t>Dự án / Squad</t>
-  </si>
-  <si>
-    <t>Người đánh giá</t>
-  </si>
-  <si>
-    <t>Nhóm năng lực</t>
-  </si>
-  <si>
-    <t>Trọng số (%)</t>
-  </si>
-  <si>
-    <t>Điểm (1–5)</t>
-  </si>
-  <si>
-    <t>Điểm quy đổi</t>
-  </si>
-  <si>
-    <t>Nhận xét</t>
-  </si>
-  <si>
-    <t>A. Năng lực kỹ thuật</t>
-  </si>
-  <si>
-    <t>B. Ownership &amp; trách nhiệm</t>
-  </si>
-  <si>
-    <t>C. DevOps &amp; vận hành (bắt buộc)</t>
-  </si>
-  <si>
-    <t>D. AI Agent &amp; cải tiến (bắt buộc)</t>
-  </si>
-  <si>
-    <t>TỔNG P2</t>
-  </si>
-  <si>
-    <t>THANG ĐÁNH GIÁ CHI TIẾT (1–5)</t>
-  </si>
-  <si>
-    <t>Mức</t>
-  </si>
-  <si>
-    <t>Mô tả</t>
-  </si>
-  <si>
-    <t>Phải được hướng dẫn để làm được; còn phụ thuộc người khác; dễ sai sót.</t>
-  </si>
-  <si>
-    <t>Làm được phần việc rõ ràng; cần review sát; chất lượng chưa ổn định.</t>
-  </si>
-  <si>
-    <t>Chủ động hoàn thành; chất lượng ổn; debug/hoàn thiện độc lập trong phạm vi.</t>
-  </si>
-  <si>
-    <t>Làm tốt và ổn định; ít rework; chủ động xử lý rủi ro, nâng chất lượng.</t>
-  </si>
-  <si>
-    <t>Extra: làm vượt kỳ vọng; tối ưu/chuẩn hoá; hướng dẫn người khác, lan toả best-practice.</t>
-  </si>
-  <si>
-    <t>Phần này phản ánh kết quả đầu ra, không đánh giá lại năng lực hay cách làm việc. (P2-Core là phần đánh giá NĂNG LỰC &amp; CÁCH LÀM VIỆC mang tính nền tảng và dài hạn của nhân sự Công Nghệ.)</t>
-  </si>
-  <si>
-    <t>Tiêu chí</t>
-  </si>
-  <si>
-    <t>Mức độ hoàn thành OKR</t>
-  </si>
-  <si>
-    <t>Tỷ lệ hoàn thành các mục tiêu đã cam kết trong kỳ đánh giá</t>
-  </si>
-  <si>
-    <t>Chất lượng kết quả</t>
-  </si>
-  <si>
-    <t>Ít lỗi nghiêm trọng; hạn chế làm lại; không gây rủi ro hệ thống</t>
-  </si>
-  <si>
-    <t>Cam kết &amp; tiến độ</t>
-  </si>
-  <si>
-    <t>Hoàn thành đúng hạn; chủ động báo sớm rủi ro; phối hợp tốt</t>
-  </si>
-  <si>
-    <t>P2-Delivery</t>
-  </si>
-  <si>
-    <t>MÔ TẢ NĂNG LỰC THEO VAI TRÒ</t>
-  </si>
-  <si>
-    <t>Gợi ý: dùng nút +/- (Outline) để thu gọn/mở rộng theo từng Vai trò. Cấp độ 1 (Thực thi – phối hợp): Làm tốt phần việc kỹ thuật của mình | Cấp độ 2 (Chủ động – cải tiến): Giải quyết bài toán xuyên hệ thống | Cấp độ 3 (Chuẩn hoá – dẫn dắt): Định hướng, tạo chuẩn, mở rộng</t>
-  </si>
-  <si>
-    <t>Backend</t>
-  </si>
-  <si>
-    <t>Cấp độ 1</t>
-  </si>
-  <si>
-    <t>Cấp độ 2</t>
-  </si>
-  <si>
-    <t>Cấp độ 3</t>
-  </si>
-  <si>
-    <t>Tự triển khai tính năng (API + DB); code dễ đọc; tests cơ bản; xử lý trường hợp lỗi không mong muốn xảy ra.</t>
-  </si>
-  <si>
-    <t>Thiết kế kiến trúc/module gọn; cải thiện performance/security; tests chắc; nâng chất lượng qua review.</t>
-  </si>
-  <si>
-    <t>Định hướng kiến trúc hệ thống có khả năng mở rộng; chủ động ngăn ngừa rủi ro và lỗi hệ thống; dẫn dắt cải tiến kỹ thuật lớn và hỗ trợ nâng cao năng lực đội ngũ.</t>
-  </si>
-  <si>
-    <t>Bàn giao công việc ổn định; biết tách công việc thành các đầu việc rõ ràng; chịu trách nhiệm xử lý lỗi đến khi hoàn tất; chủ động báo sớm các rủi ro phát sinh.</t>
-  </si>
-  <si>
-    <t>Chủ động quản lý phạm vi và rủi ro công việc; phối hợp hiệu quả với các bộ phận liên quan; giảm phát sinh làm lại nhờ yêu cầu và tài liệu được chuẩn bị rõ ràng.</t>
-  </si>
-  <si>
-    <t>Cải tiến quy trình bàn giao công việc trong đội (tiêu chí hoàn thành, danh sách rà soát); xử lý các điểm nghẽn trong phối hợp giữa các nhóm; nâng cao khả năng dự báo và kiểm soát tiến độ chung.</t>
-  </si>
-  <si>
-    <t>C. DevOps &amp; vận hành</t>
-  </si>
-  <si>
-    <t>Thực hiện quy trình tích hợp và triển khai tự động; hiểu và sử dụng đúng cấu hình môi trường, thông tin bảo mật; theo dõi nhật ký và lỗi hệ thống; tham gia trực xử lý sự cố khi cần.</t>
-  </si>
-  <si>
-    <t>Chủ động cải thiện quy trình triển khai (tối ưu hiệu năng, kiểm soát chất lượng); bổ sung theo dõi chỉ số và cảnh báo; thực hiện phương án quay lui khi có sự cố; nâng cao độ ổn định và rút ngắn thời gian khắc phục lỗi.</t>
-  </si>
-  <si>
-    <t>Chuẩn hóa quy trình phát hành và giám sát hệ thống; xây dựng hướng dẫn vận hành và xử lý sự cố; chủ trì phân tích nguyên nhân sau sự cố; hướng dẫn và nâng cao năng lực vận hành cho đội ngũ.</t>
-  </si>
-  <si>
-    <t>D. AI Agent &amp; cải tiến</t>
-  </si>
-  <si>
-    <t>Sử dụng AI Agent để hỗ trợ code, chỉnh sửa code, viết kiểm thử và tìm lỗi; biết đặt yêu cầu rõ ràng; luôn kiểm tra lại kết quả trước khi áp dụng.</t>
-  </si>
-  <si>
-    <t>Xây dựng mẫu yêu cầu và quy trình làm việc có thể tái sử dụng; dùng AI để hỗ trợ rà soát và tìm lỗi; theo dõi hiệu quả bằng các chỉ số như thời gian hoàn thành và tỷ lệ lỗi phát sinh.</t>
-  </si>
-  <si>
-    <t>Dẫn dắt việc áp dụng AI trong kỹ thuật một cách có kiểm soát; đào tạo và hướng dẫn đội ngũ; tự động hóa các công việc lặp lại theo nguyên tắc an toàn, phân quyền và tuân thủ quy định nội bộ.</t>
-  </si>
-  <si>
-    <t>Designer</t>
-  </si>
-  <si>
-    <t>Tự xây dựng luồng trải nghiệm và đặc tả giao diện; đảm bảo tính nhất quán về hình ảnh; bàn giao thiết kế rõ ràng để đội triển khai chính xác.</t>
-  </si>
-  <si>
-    <t>Cải thiện khả năng sử dụng dựa trên nghiên cứu và đánh giá trải nghiệm; phát triển và mở rộng hệ thống thiết kế; giảm phát sinh làm lại nhờ đặc tả thiết kế rõ ràng.</t>
-  </si>
-  <si>
-    <t>Định hướng thiết kế tổng thể; tạo ra tác động trải nghiệm người dùng có thể đo lường; quản trị và chuẩn hóa hệ thống thiết kế; hướng dẫn và kết nối các đội cùng áp dụng.</t>
-  </si>
-  <si>
-    <t>Bàn giao công việc ổn định; xác định rõ phạm vi; lặp lại thiết kế kịp thời; phối hợp sớm với các bên triển khai để thống nhất ràng buộc.</t>
-  </si>
-  <si>
-    <t>Quản lý các lựa chọn và đánh đổi trong thiết kế; chuẩn bị phương án thay thế; ghi nhận rõ các quyết định; giảm phát sinh làm lại thông qua rà soát thiết kế.</t>
-  </si>
-  <si>
-    <t>Nâng chuẩn bàn giao thiết kế (tiêu chí hoàn thành, danh sách rà soát); tháo gỡ các vướng mắc phối hợp giữa các đội; nâng cao khả năng dự báo và kiểm soát tiến độ.</t>
-  </si>
-  <si>
-    <t>Làm việc với môi trường preview và staging; sử dụng nhất quán các thành phần và chuẩn thiết kế; xây dựng đặc tả phù hợp với khả năng triển khai.</t>
-  </si>
-  <si>
-    <t>Thúc đẩy áp dụng chuẩn thành phần thiết kế; cải thiện tự động hóa bàn giao thiết kế–triển khai; giảm lỗi tích hợp và công việc làm lại.</t>
-  </si>
-  <si>
-    <t>Dẫn dắt chuẩn hóa quy trình thiết kế–triển khai với đội phát triển; xây dựng hướng dẫn và các thực hành tốt cho toàn đội.</t>
-  </si>
-  <si>
-    <t>Sử dụng AI để hỗ trợ xây dựng khung thiết kế, nội dung trải nghiệm và phương án thiết kế; biết đặt yêu cầu phù hợp; kiểm tra và đối chiếu với hệ thống thiết kế hiện có.</t>
-  </si>
-  <si>
-    <t>Xây dựng thư viện yêu cầu AI có thể tái sử dụng; tăng tốc tổng hợp nghiên cứu; theo dõi tác động của AI đến thời gian thực hiện và mức độ làm lại.</t>
-  </si>
-  <si>
-    <t>Dẫn dắt việc áp dụng AI trong thiết kế một cách an toàn và có kiểm soát; đào tạo đội ngũ; tự động hóa các công việc lặp lại theo quy định và chuẩn quản trị.</t>
-  </si>
-  <si>
-    <t>FrontEnd</t>
-  </si>
-  <si>
-    <t>Tự triển khai tính năng giao diện từ đầu đến cuối (giao diện, trạng thái, tích hợp dữ liệu); xử lý các tình huống phát sinh; viết mã rõ ràng, dễ bảo trì.</t>
-  </si>
-  <si>
-    <t>Cải thiện hiệu năng và khả năng truy cập của giao diện; xây dựng thành phần dùng lại; nâng cao kiến trúc và kiểm thử để tăng độ ổn định.</t>
-  </si>
-  <si>
-    <t>Định hướng kỹ thuật frontend; dẫn dắt các thay đổi lớn để giảm rủi ro; hướng dẫn đội ngũ; chủ động ngăn ngừa lỗi ảnh hưởng diện rộng trên giao diện.</t>
-  </si>
-  <si>
-    <t>Bàn giao công việc ổn định; chịu trách nhiệm xử lý lỗi đến khi hoàn tất; phối hợp sớm với backend và thiết kế; chủ động báo rủi ro.</t>
-  </si>
-  <si>
-    <t>Quản lý các lựa chọn và đánh đổi về trải nghiệm người dùng; giảm phát sinh làm lại; nâng chất lượng bàn giao bằng đặc tả, minh chứng và tài liệu rõ ràng.</t>
-  </si>
-  <si>
-    <t>Nâng chuẩn bàn giao và rà soát (chuẩn thành phần, danh sách rà soát); tháo gỡ vướng mắc phối hợp giữa các đội; nâng cao khả năng dự báo và kiểm soát tiến độ.</t>
-  </si>
-  <si>
-    <t>Sử dụng thành thạo quy trình tích hợp và triển khai; quản lý cấu hình môi trường; theo dõi lỗi phía người dùng; giữ bản phát hành gọn và ổn định.</t>
-  </si>
-  <si>
-    <t>Cải thiện quy trình triển khai (tối ưu tốc độ, kiểm soát chất lượng); giảm kích thước và thời gian tải; có phương án quay lui khi sự cố; nâng cao độ ổn định.</t>
-  </si>
-  <si>
-    <t>Chuẩn hóa phát hành và giám sát cho frontend; xây dựng hướng dẫn xử lý sự cố; hướng dẫn đội ngũ thực hành vận hành; giảm lỗi phía người dùng và rút ngắn thời gian khắc phục.</t>
-  </si>
-  <si>
-    <t>Sử dụng AI để hỗ trợ tạo khung code, chỉnh sửa code, viết kiểm thử và tìm lỗi; biết đặt yêu cầu rõ ràng; luôn kiểm tra lại trước khi áp dụng.</t>
-  </si>
-  <si>
-    <t>Xây dựng mẫu yêu cầu AI có thể tái sử dụng (thành phần, khả năng truy cập, kiểm thử); dùng AI hỗ trợ rà soát và cải tiến mã; theo dõi hiệu quả bằng các chỉ số phù hợp.</t>
-  </si>
-  <si>
-    <t>Dẫn dắt việc áp dụng AI trong frontend theo quy chuẩn; đào tạo đội ngũ; tự động hóa các công việc lặp lại một cách an toàn và có kiểm soát.</t>
-  </si>
-  <si>
-    <t>FullStack</t>
-  </si>
-  <si>
-    <t>Tự triển khai tính năng từ đầu đến cuối (giao diện, xử lý dữ liệu, lưu trữ); đảm bảo chất lượng cơ bản; viết kiểm thử cần thiết; xử lý các tình huống lỗi phát sinh.</t>
-  </si>
-  <si>
-    <t>Phân định rõ trách nhiệm giữa backend và frontend; cải thiện hiệu năng và an toàn hệ thống; thực hiện tái cấu trúc có kiểm soát; xây dựng kiểm thử vững chắc hơn.</t>
-  </si>
-  <si>
-    <t>Định hướng kỹ thuật end-to-end; chủ động ngăn ngừa rủi ro và lỗi hệ thống; hướng dẫn đội ngũ; dẫn dắt các đợt tái cấu trúc và chuyển đổi hệ thống lớn một cách an toàn.</t>
-  </si>
-  <si>
-    <t>Chịu trách nhiệm toàn bộ tính năng từ đầu đến cuối; đảm bảo vận hành ổn định; chủ động báo rủi ro; xử lý triệt để vấn đề đến khi hoàn tất.</t>
-  </si>
-  <si>
-    <t>Quản lý phạm vi và rủi ro công việc; trao đổi và thống nhất các đánh đổi kỹ thuật; giảm phát sinh làm lại; cải thiện chất lượng tài liệu và bàn giao.</t>
-  </si>
-  <si>
-    <t>Nâng cao khả năng dự báo; xây dựng và áp dụng các chuẩn chung (tiêu chí hoàn thành, danh sách rà soát); tháo gỡ vướng mắc trong phối hợp giữa các đội.</t>
-  </si>
-  <si>
-    <t>Sử dụng quy trình tích hợp và triển khai tự động; quản lý cấu hình và thông tin bảo mật; theo dõi lỗi và nhật ký hệ thống; triển khai an toàn và tham gia trực xử lý sự cố.</t>
-  </si>
-  <si>
-    <t>Cải thiện quy trình triển khai; bổ sung theo dõi chỉ số và cảnh báo; có phương án quay lui khi cần; nâng cao độ ổn định trên toàn bộ hệ thống.</t>
-  </si>
-  <si>
-    <t>Chuẩn hóa phát hành và giám sát hệ thống; xây dựng hướng dẫn vận hành và xử lý sự cố; giảm thời gian khắc phục lỗi; hướng dẫn đội ngũ thực hành vận hành hiệu quả.</t>
-  </si>
-  <si>
-    <t>Sử dụng AI hỗ trợ toàn bộ chuỗi phát triển (tạo khung, chỉnh sửa code, kiểm thử, tìm lỗi); biết đặt yêu cầu phù hợp; luôn rà soát kỹ kết quả trước khi áp dụng.</t>
-  </si>
-  <si>
-    <t>Xây dựng mẫu yêu cầu và quy trình làm việc với AI có thể tái sử dụng; dùng AI hỗ trợ rà soát và tìm lỗi; theo dõi tác động đến thời gian thực hiện và chất lượng.</t>
-  </si>
-  <si>
-    <t>Dẫn dắt việc áp dụng AI trong phát triển end-to-end một cách an toàn và có kiểm soát; đào tạo đội ngũ; tự động hóa các công việc xuyên suốt theo chuẩn quản trị.</t>
-  </si>
-  <si>
-    <t>Kết quả công việc (P2-Delivery – từ OKR/KPI)</t>
-  </si>
-  <si>
-    <t>P2-Delivery = Trung bình cộng các tiêu chí trên</t>
-  </si>
-  <si>
-    <t>P2+ là mô hình đánh giá năng lực mở rộng, trong đó kết quả thực hiện OKR/KPI được tích hợp như một thành phần của P2, thay vì tách thành P3 độc lập. Mục tiêu là đơn giản hóa quy trình, phản ánh đúng đặc thù công việc kỹ thuật và đảm bảo đánh giá cân bằng giữa năng lực dài hạn và kết quả ngắn hạn.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -604,14 +607,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -708,7 +703,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -720,30 +715,6 @@
       <left style="thin">
         <color rgb="FFC9CDD2"/>
       </left>
-      <right style="thin">
-        <color rgb="FFC9CDD2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFC9CDD2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFC9CDD2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFC9CDD2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFC9CDD2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color rgb="FFC9CDD2"/>
       </right>
@@ -801,19 +772,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -826,11 +784,163 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC9CDD2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC9CDD2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC9CDD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -853,40 +963,63 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -897,49 +1030,91 @@
     <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -949,28 +1124,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1008,13 +1161,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFBBF7D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFDCFCE7"/>
         </patternFill>
       </fill>
@@ -1037,6 +1183,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFBBF7D0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1316,40 +1469,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="50" t="s">
-        <v>149</v>
-      </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
+      <c r="A3" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
     </row>
     <row r="5" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
+      <c r="A5" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
+      <c r="A6" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1372,286 +1525,296 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
+      <c r="A1" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="3" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="A3" s="54" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
     </row>
     <row r="4" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
+      <c r="A4" s="38" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="35"/>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
+      <c r="A5" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="35"/>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="30"/>
+      <c r="D6" s="35"/>
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
+      <c r="A7" s="27"/>
+      <c r="B7" s="39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="30"/>
+      <c r="D7" s="35"/>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="30"/>
+      <c r="D8" s="35"/>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="45"/>
+      <c r="D9" s="46"/>
     </row>
     <row r="11" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
+      <c r="A11" s="51" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="43"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="28" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
+      <c r="A12" s="27"/>
+      <c r="B12" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="30"/>
+      <c r="D12" s="35"/>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="45"/>
+      <c r="D13" s="46"/>
     </row>
     <row r="16" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
+      <c r="A16" s="54" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="43"/>
     </row>
     <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
+      <c r="A17" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="35"/>
     </row>
     <row r="18" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
+      <c r="A18" s="55" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="46"/>
     </row>
     <row r="19" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
+      <c r="A19" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
     </row>
     <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
+      <c r="A20" s="40" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
+      <c r="A21" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
     </row>
     <row r="23" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
+      <c r="A23" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
     </row>
     <row r="24" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
+      <c r="A24" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="43"/>
     </row>
     <row r="25" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
+      <c r="A25" s="27"/>
+      <c r="B25" s="52" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="30"/>
+      <c r="D25" s="35"/>
     </row>
     <row r="26" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
+      <c r="A26" s="27"/>
+      <c r="B26" s="52" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="30"/>
+      <c r="D26" s="35"/>
     </row>
     <row r="27" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" s="45"/>
+      <c r="D27" s="46"/>
     </row>
     <row r="29" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
+      <c r="A29" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="43"/>
     </row>
     <row r="30" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="45"/>
+      <c r="D30" s="46"/>
     </row>
     <row r="32" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
+      <c r="A32" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32" s="42"/>
+      <c r="C32" s="42"/>
+      <c r="D32" s="43"/>
     </row>
     <row r="33" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
+      <c r="A33" s="27"/>
+      <c r="B33" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="C33" s="30"/>
+      <c r="D33" s="35"/>
     </row>
     <row r="34" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
+      <c r="A34" s="28"/>
+      <c r="B34" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" s="45"/>
+      <c r="D34" s="46"/>
     </row>
     <row r="37" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="B37" s="21"/>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
+      <c r="A37" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="50"/>
     </row>
     <row r="38" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="15" t="s">
+      <c r="A38" s="14" t="s">
         <v>32</v>
       </c>
+      <c r="B38" s="14" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="39" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="B39" s="16" t="s">
+      <c r="A39" s="15" t="s">
         <v>34</v>
       </c>
+      <c r="B39" s="15" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="40" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B40" s="16" t="s">
+      <c r="A40" s="15" t="s">
         <v>36</v>
       </c>
+      <c r="B40" s="15" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="41" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B41" s="16" t="s">
+      <c r="A41" s="15" t="s">
         <v>38</v>
       </c>
+      <c r="B41" s="15" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="42" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B42" s="16" t="s">
+      <c r="A42" s="15" t="s">
         <v>40</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="B12:D12"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="B30:D30"/>
-    <mergeCell ref="A11:D11"/>
     <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A20:D20"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1659,7 +1822,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1671,112 +1834,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
+      <c r="A1" s="62" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="60"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="33"/>
+      <c r="E3" s="60"/>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="21"/>
+        <v>45</v>
+      </c>
+      <c r="B4" s="60"/>
+      <c r="C4" s="30"/>
       <c r="D4" s="5" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="E4" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B7" s="3">
         <v>35</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3" t="str">
-        <f>IF(C7="","",B7*C7/100)</f>
+        <f>IF(C7="","",B7*IF(C7="L1",1.5,IF(C7="L2",3.5,IF(C7="L3",5,0)))/100)</f>
         <v/>
       </c>
       <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="B8" s="3">
         <v>25</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="str">
-        <f>IF(C8="","",B8*C8/100)</f>
+        <f>IF(C8="","",B8*IF(C8="L1",1.5,IF(C8="L2",3.5,IF(C8="L3",5,0)))/100)</f>
         <v/>
       </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="B9" s="3">
         <v>20</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="str">
-        <f>IF(C9="","",B9*C9/100)</f>
+        <f>IF(C9="","",B9*IF(C9="L1",1.5,IF(C9="L2",3.5,IF(C9="L3",5,0)))/100)</f>
         <v/>
       </c>
       <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="B10" s="3">
         <v>20</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="str">
-        <f>IF(C10="","",B10*C10/100)</f>
+        <f>IF(C10="","",B10*IF(C10="L1",1.5,IF(C10="L2",3.5,IF(C10="L3",5,0)))/100)</f>
         <v/>
       </c>
       <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B11" s="6">
         <v>100</v>
@@ -1789,214 +1952,213 @@
       <c r="E11" s="7"/>
     </row>
     <row r="13" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="64" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="66" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+    </row>
+    <row r="15" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="58"/>
+    </row>
+    <row r="16" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="58"/>
+    </row>
+    <row r="17" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="58"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="21"/>
+      <c r="B18" s="22"/>
+    </row>
+    <row r="21" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" s="57"/>
+      <c r="C21" s="58"/>
+    </row>
+    <row r="22" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="61" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="57"/>
+      <c r="C22" s="58"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="26"/>
+    </row>
+    <row r="24" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="C25" s="18"/>
+    </row>
+    <row r="26" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B26" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="37"/>
-    </row>
-    <row r="15" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8">
-        <v>1</v>
-      </c>
-      <c r="B15" s="35" t="s">
+      <c r="C26" s="18"/>
+    </row>
+    <row r="27" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-    </row>
-    <row r="16" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8">
-        <v>2</v>
-      </c>
-      <c r="B16" s="35" t="s">
+      <c r="B27" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="37"/>
-    </row>
-    <row r="17" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8">
-        <v>3</v>
-      </c>
-      <c r="B17" s="35" t="s">
+      <c r="C27" s="18"/>
+    </row>
+    <row r="29" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="65" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-    </row>
-    <row r="18" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8">
-        <v>4</v>
-      </c>
-      <c r="B18" s="35" t="s">
+      <c r="B29" s="57"/>
+      <c r="C29" s="58"/>
+    </row>
+    <row r="30" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
-    </row>
-    <row r="19" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8">
-        <v>5</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-    </row>
-    <row r="22" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="43" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="30" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-    </row>
-    <row r="24" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="C25" s="19"/>
-    </row>
-    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" s="19"/>
-    </row>
-    <row r="27" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="C27" s="19"/>
-    </row>
-    <row r="29" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="44" t="s">
-        <v>148</v>
-      </c>
-      <c r="B29" s="45"/>
-      <c r="C29" s="45"/>
-    </row>
-    <row r="30" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="46" t="s">
-        <v>87</v>
-      </c>
-      <c r="B30" s="48" t="str">
-        <f>IF(COUNT(C25:C27)=0,"",AVERAGE(C25:C27))</f>
-        <v/>
-      </c>
-      <c r="C30" s="49"/>
+      <c r="B30" s="59" t="str">
+        <f>IF(COUNTA(C25:C27)=0,"",
+AVERAGE(
+ IF(C25="Chưa đạt",1.5,IF(C25="Đạt",3.5,IF(C25="Tốt",5,""))),
+ IF(C26="Chưa đạt",1.5,IF(C26="Đạt",3.5,IF(C26="Tốt",5,""))),
+ IF(C27="Chưa đạt",1.5,IF(C27="Đạt",3.5,IF(C27="Tốt",5,"")))
+))</f>
+        <v/>
+      </c>
+      <c r="C30" s="58"/>
     </row>
     <row r="31" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" s="48" t="str">
-        <f>IF(OR(D11="",B30=""),"",D11*0.7 + B30*0.3)</f>
-        <v/>
-      </c>
-      <c r="C31" s="49"/>
+      <c r="A31" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="59" t="str">
+        <f>IF(OR(D11="",B30=""),"",D11*0.5+B30*0.5)</f>
+        <v/>
+      </c>
+      <c r="C31" s="58"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="B30:C30"/>
+  <mergeCells count="14">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B19:E19"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3"/>
+    <mergeCell ref="A22:C22"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B15:E15"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C10">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="3" operator="equal">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="between">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="between">
       <formula>2.5</formula>
       <formula>3.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="8" operator="between">
+    <cfRule type="cellIs" dxfId="5" priority="8" operator="between">
       <formula>3.3</formula>
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="9" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="C7:C10" xr:uid="{00000000-0002-0000-0200-000000000000}">
+      <formula1>"L1,L2,L3"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="C25:C27" xr:uid="{00000000-0002-0000-0200-000001000000}">
+      <formula1>"Chưa đạt,Đạt,Tốt"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr applyStyles="1" summaryBelow="0"/>
   </sheetPr>
@@ -2008,331 +2170,331 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="67" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+    </row>
+    <row r="2" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="69" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+    </row>
+    <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="68" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+    </row>
+    <row r="5" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-    </row>
-    <row r="2" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
+      <c r="D7" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-    </row>
-    <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-    </row>
-    <row r="5" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="9" t="s">
+      <c r="B8" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C8" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D8" s="11" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" s="11" t="s">
+    <row r="9" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="B9" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="C9" s="11" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="12" t="s">
+      <c r="D9" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="12" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+    </row>
+    <row r="12" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="D13" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="12" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="C14" s="11" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
+      <c r="D14" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="12" t="s">
+    </row>
+    <row r="15" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C15" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D15" s="11" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="41" t="s">
+    <row r="16" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-    </row>
-    <row r="12" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B13" s="12" t="s">
+      <c r="C16" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="D16" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D13" s="12" t="s">
+    </row>
+    <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="68" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B14" s="12" t="s">
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+    </row>
+    <row r="19" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D20" s="11" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="B15" s="12" t="s">
+    <row r="21" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C21" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D21" s="11" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="B16" s="12" t="s">
+    <row r="22" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C22" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D22" s="11" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="41" t="s">
+    <row r="23" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-    </row>
-    <row r="19" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B20" s="12" t="s">
+      <c r="C23" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="D23" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="D20" s="12" t="s">
+    </row>
+    <row r="25" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="68" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B21" s="12" t="s">
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+    </row>
+    <row r="26" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C27" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D27" s="11" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="B22" s="12" t="s">
+    <row r="28" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C28" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D28" s="11" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="B23" s="12" t="s">
+    <row r="29" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B29" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C29" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D29" s="11" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="41" t="s">
+    <row r="30" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-    </row>
-    <row r="26" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B27" s="12" t="s">
+      <c r="C30" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="D30" s="11" t="s">
         <v>136</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2355,7 +2517,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:N35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2371,71 +2533,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="A1" s="62" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
+      <c r="A3" s="60" t="s">
+        <v>138</v>
+      </c>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
     </row>
     <row r="5" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>47</v>
+        <v>140</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="J5" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="K5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="L5" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="M5" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="N5" s="17" t="s">
-        <v>31</v>
+      <c r="L5" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="M5" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="N5" s="16" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -2443,10 +2605,10 @@
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>52</v>
+        <v>145</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>53</v>
+        <v>146</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -2459,19 +2621,19 @@
         <v/>
       </c>
       <c r="H6" s="4"/>
-      <c r="J6" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K6" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M6" s="14" t="str">
+      <c r="J6" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K6" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M6" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N6" s="14" t="str">
+      <c r="N6" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2481,10 +2643,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>54</v>
+        <v>147</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>55</v>
+        <v>148</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -2497,19 +2659,19 @@
         <v/>
       </c>
       <c r="H7" s="4"/>
-      <c r="J7" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K7" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M7" s="14" t="str">
+      <c r="J7" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K7" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M7" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N7" s="14" t="str">
+      <c r="N7" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2519,10 +2681,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>56</v>
+        <v>149</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>55</v>
+        <v>148</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
@@ -2535,19 +2697,19 @@
         <v/>
       </c>
       <c r="H8" s="4"/>
-      <c r="J8" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K8" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M8" s="14" t="str">
+      <c r="J8" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K8" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M8" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N8" s="14" t="str">
+      <c r="N8" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2557,10 +2719,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
+        <v>150</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>55</v>
+        <v>148</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -2573,19 +2735,19 @@
         <v/>
       </c>
       <c r="H9" s="4"/>
-      <c r="J9" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K9" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M9" s="14" t="str">
+      <c r="J9" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K9" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M9" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N9" s="14" t="str">
+      <c r="N9" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2607,19 +2769,19 @@
         <v/>
       </c>
       <c r="H10" s="4"/>
-      <c r="J10" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K10" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M10" s="14" t="str">
+      <c r="J10" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K10" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M10" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N10" s="14" t="str">
+      <c r="N10" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2641,19 +2803,19 @@
         <v/>
       </c>
       <c r="H11" s="4"/>
-      <c r="J11" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K11" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M11" s="14" t="str">
+      <c r="J11" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K11" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M11" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N11" s="14" t="str">
+      <c r="N11" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2675,19 +2837,19 @@
         <v/>
       </c>
       <c r="H12" s="4"/>
-      <c r="J12" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K12" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M12" s="14" t="str">
+      <c r="J12" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K12" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M12" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N12" s="14" t="str">
+      <c r="N12" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2709,19 +2871,19 @@
         <v/>
       </c>
       <c r="H13" s="4"/>
-      <c r="J13" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K13" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M13" s="14" t="str">
+      <c r="J13" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K13" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M13" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N13" s="14" t="str">
+      <c r="N13" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2743,19 +2905,19 @@
         <v/>
       </c>
       <c r="H14" s="4"/>
-      <c r="J14" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K14" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M14" s="14" t="str">
+      <c r="J14" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K14" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M14" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N14" s="14" t="str">
+      <c r="N14" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2777,19 +2939,19 @@
         <v/>
       </c>
       <c r="H15" s="4"/>
-      <c r="J15" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K15" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M15" s="14" t="str">
+      <c r="J15" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K15" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M15" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N15" s="14" t="str">
+      <c r="N15" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2811,19 +2973,19 @@
         <v/>
       </c>
       <c r="H16" s="4"/>
-      <c r="J16" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K16" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M16" s="14" t="str">
+      <c r="J16" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K16" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M16" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N16" s="14" t="str">
+      <c r="N16" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2845,19 +3007,19 @@
         <v/>
       </c>
       <c r="H17" s="4"/>
-      <c r="J17" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K17" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M17" s="14" t="str">
+      <c r="J17" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K17" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M17" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N17" s="14" t="str">
+      <c r="N17" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2879,19 +3041,19 @@
         <v/>
       </c>
       <c r="H18" s="4"/>
-      <c r="J18" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K18" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M18" s="14" t="str">
+      <c r="J18" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K18" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M18" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N18" s="14" t="str">
+      <c r="N18" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2913,19 +3075,19 @@
         <v/>
       </c>
       <c r="H19" s="4"/>
-      <c r="J19" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K19" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M19" s="14" t="str">
+      <c r="J19" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K19" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M19" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N19" s="14" t="str">
+      <c r="N19" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2947,19 +3109,19 @@
         <v/>
       </c>
       <c r="H20" s="4"/>
-      <c r="J20" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K20" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M20" s="14" t="str">
+      <c r="J20" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K20" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M20" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N20" s="14" t="str">
+      <c r="N20" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -2981,19 +3143,19 @@
         <v/>
       </c>
       <c r="H21" s="4"/>
-      <c r="J21" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K21" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M21" s="14" t="str">
+      <c r="J21" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K21" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M21" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N21" s="14" t="str">
+      <c r="N21" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3015,19 +3177,19 @@
         <v/>
       </c>
       <c r="H22" s="4"/>
-      <c r="J22" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K22" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M22" s="14" t="str">
+      <c r="J22" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K22" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M22" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N22" s="14" t="str">
+      <c r="N22" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3049,19 +3211,19 @@
         <v/>
       </c>
       <c r="H23" s="4"/>
-      <c r="J23" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K23" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M23" s="14" t="str">
+      <c r="J23" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K23" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M23" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N23" s="14" t="str">
+      <c r="N23" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3083,19 +3245,19 @@
         <v/>
       </c>
       <c r="H24" s="4"/>
-      <c r="J24" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K24" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M24" s="14" t="str">
+      <c r="J24" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K24" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M24" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N24" s="14" t="str">
+      <c r="N24" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3117,19 +3279,19 @@
         <v/>
       </c>
       <c r="H25" s="4"/>
-      <c r="J25" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K25" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M25" s="14" t="str">
+      <c r="J25" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K25" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M25" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N25" s="14" t="str">
+      <c r="N25" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3151,19 +3313,19 @@
         <v/>
       </c>
       <c r="H26" s="4"/>
-      <c r="J26" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K26" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M26" s="14" t="str">
+      <c r="J26" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K26" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M26" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N26" s="14" t="str">
+      <c r="N26" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3185,19 +3347,19 @@
         <v/>
       </c>
       <c r="H27" s="4"/>
-      <c r="J27" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K27" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M27" s="14" t="str">
+      <c r="J27" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K27" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M27" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N27" s="14" t="str">
+      <c r="N27" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3219,19 +3381,19 @@
         <v/>
       </c>
       <c r="H28" s="4"/>
-      <c r="J28" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K28" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M28" s="14" t="str">
+      <c r="J28" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K28" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M28" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N28" s="14" t="str">
+      <c r="N28" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3253,19 +3415,19 @@
         <v/>
       </c>
       <c r="H29" s="4"/>
-      <c r="J29" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K29" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M29" s="14" t="str">
+      <c r="J29" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K29" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M29" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N29" s="14" t="str">
+      <c r="N29" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3287,19 +3449,19 @@
         <v/>
       </c>
       <c r="H30" s="4"/>
-      <c r="J30" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K30" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M30" s="14" t="str">
+      <c r="J30" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K30" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M30" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N30" s="14" t="str">
+      <c r="N30" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3321,19 +3483,19 @@
         <v/>
       </c>
       <c r="H31" s="4"/>
-      <c r="J31" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K31" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M31" s="14" t="str">
+      <c r="J31" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K31" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M31" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N31" s="14" t="str">
+      <c r="N31" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3355,19 +3517,19 @@
         <v/>
       </c>
       <c r="H32" s="4"/>
-      <c r="J32" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K32" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M32" s="14" t="str">
+      <c r="J32" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K32" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M32" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N32" s="14" t="str">
+      <c r="N32" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3389,19 +3551,19 @@
         <v/>
       </c>
       <c r="H33" s="4"/>
-      <c r="J33" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K33" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M33" s="14" t="str">
+      <c r="J33" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K33" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M33" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N33" s="14" t="str">
+      <c r="N33" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3423,19 +3585,19 @@
         <v/>
       </c>
       <c r="H34" s="4"/>
-      <c r="J34" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K34" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M34" s="14" t="str">
+      <c r="J34" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K34" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M34" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N34" s="14" t="str">
+      <c r="N34" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3457,19 +3619,19 @@
         <v/>
       </c>
       <c r="H35" s="4"/>
-      <c r="J35" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K35" s="14" t="e">
-        <f>Product_Engineer!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M35" s="14" t="str">
+      <c r="J35" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K35" s="13" t="e">
+        <f>Product_Engineer!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M35" s="13" t="str">
         <f>Product_Engineer!B30</f>
         <v/>
       </c>
-      <c r="N35" s="14" t="str">
+      <c r="N35" s="13" t="str">
         <f>Product_Engineer!B31</f>
         <v/>
       </c>
@@ -3480,18 +3642,18 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:E35">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="between">
       <formula>2.5</formula>
       <formula>3.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="between">
       <formula>3.3</formula>
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Add new member-specific Excel files for P2 project, including forms for Chuong, Dat, Duc, Ho, and Hoang. Update existing P2_Form_BP_Cong_Nghe.xlsx for consistency.
</commit_message>
<xml_diff>
--- a/P2_Form_BP_Cong_Nghe.xlsx
+++ b/P2_Form_BP_Cong_Nghe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CONG VIEC\project-management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA7B0945-FC5E-4FF5-94C5-AD2D5FCA2E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0366F2-F97C-4BBF-8E91-5449CFA42C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="182">
   <si>
     <t>CẤU TRÚC &amp; TRỌNG SỐ P2+</t>
   </si>
@@ -583,6 +583,9 @@
   </si>
   <si>
     <t>VAI TRÒ</t>
+  </si>
+  <si>
+    <t>NGUYỄN HUY HOÀNG</t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1076,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1195,108 +1198,27 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1325,6 +1247,87 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1344,6 +1347,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1699,40 +1703,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="66" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
     </row>
     <row r="3" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
     </row>
     <row r="5" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
     </row>
     <row r="6" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="65" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1756,240 +1760,240 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="75" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
     </row>
     <row r="3" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="70" t="s">
+      <c r="A3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="61"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="72"/>
     </row>
     <row r="4" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="49"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="74"/>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="48" t="s">
+      <c r="A5" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="49"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="74"/>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13"/>
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="44"/>
-      <c r="D6" s="49"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="74"/>
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13"/>
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="49"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="74"/>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="73" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="44"/>
-      <c r="D8" s="49"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="74"/>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14"/>
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="56"/>
-      <c r="D9" s="57"/>
+      <c r="C9" s="77"/>
+      <c r="D9" s="78"/>
     </row>
     <row r="11" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="61"/>
+      <c r="B11" s="51"/>
+      <c r="C11" s="51"/>
+      <c r="D11" s="72"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="44"/>
-      <c r="D12" s="49"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="74"/>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14"/>
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="83" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="56"/>
-      <c r="D13" s="57"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="78"/>
     </row>
     <row r="16" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="70" t="s">
+      <c r="A16" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="61"/>
+      <c r="B16" s="51"/>
+      <c r="C16" s="51"/>
+      <c r="D16" s="72"/>
     </row>
     <row r="17" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="50" t="s">
+      <c r="A17" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="49"/>
+      <c r="B17" s="64"/>
+      <c r="C17" s="64"/>
+      <c r="D17" s="74"/>
     </row>
     <row r="18" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="71" t="s">
+      <c r="A18" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="56"/>
-      <c r="C18" s="56"/>
-      <c r="D18" s="57"/>
+      <c r="B18" s="77"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="78"/>
     </row>
     <row r="19" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="58" t="s">
+      <c r="A19" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
+      <c r="B19" s="64"/>
+      <c r="C19" s="64"/>
+      <c r="D19" s="64"/>
     </row>
     <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="54" t="s">
+      <c r="A20" s="82" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
+      <c r="B20" s="64"/>
+      <c r="C20" s="64"/>
+      <c r="D20" s="64"/>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="54" t="s">
+      <c r="A21" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="44"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
     </row>
     <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="51" t="s">
+      <c r="A22" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
     </row>
     <row r="24" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="63" t="s">
+      <c r="A24" s="85" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="44"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
     </row>
     <row r="25" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="59" t="s">
+      <c r="A25" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="60"/>
-      <c r="C25" s="60"/>
-      <c r="D25" s="61"/>
+      <c r="B25" s="51"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="72"/>
     </row>
     <row r="26" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>
-      <c r="B26" s="69" t="s">
+      <c r="B26" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="49"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="74"/>
     </row>
     <row r="27" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>
-      <c r="B27" s="69" t="s">
+      <c r="B27" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="44"/>
-      <c r="D27" s="49"/>
+      <c r="C27" s="64"/>
+      <c r="D27" s="74"/>
     </row>
     <row r="28" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14"/>
-      <c r="B28" s="68" t="s">
+      <c r="B28" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="C28" s="56"/>
-      <c r="D28" s="57"/>
+      <c r="C28" s="77"/>
+      <c r="D28" s="78"/>
     </row>
     <row r="30" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="59" t="s">
+      <c r="A30" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="60"/>
-      <c r="C30" s="60"/>
-      <c r="D30" s="61"/>
+      <c r="B30" s="51"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="72"/>
     </row>
     <row r="31" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14"/>
-      <c r="B31" s="68" t="s">
+      <c r="B31" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="C31" s="56"/>
-      <c r="D31" s="57"/>
+      <c r="C31" s="77"/>
+      <c r="D31" s="78"/>
     </row>
     <row r="33" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="59" t="s">
+      <c r="A33" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="B33" s="60"/>
-      <c r="C33" s="60"/>
-      <c r="D33" s="61"/>
+      <c r="B33" s="51"/>
+      <c r="C33" s="51"/>
+      <c r="D33" s="72"/>
     </row>
     <row r="34" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>
-      <c r="B34" s="69" t="s">
+      <c r="B34" s="79" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="44"/>
-      <c r="D34" s="49"/>
+      <c r="C34" s="64"/>
+      <c r="D34" s="74"/>
     </row>
     <row r="35" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="14"/>
-      <c r="B35" s="68" t="s">
+      <c r="B35" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="C35" s="56"/>
-      <c r="D35" s="57"/>
+      <c r="C35" s="77"/>
+      <c r="D35" s="78"/>
     </row>
     <row r="36" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="12"/>
     </row>
     <row r="37" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="62" t="s">
+      <c r="A37" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="56"/>
-      <c r="C37" s="56"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
+      <c r="B37" s="77"/>
+      <c r="C37" s="77"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
     </row>
     <row r="38" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="26" t="s">
@@ -2081,10 +2085,10 @@
       <c r="B43" s="37"/>
     </row>
     <row r="44" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="65" t="s">
+      <c r="A44" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="66"/>
+      <c r="B44" s="70"/>
     </row>
     <row r="45" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="25" t="s">
@@ -2236,6 +2240,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="B12:D12"/>
@@ -2252,20 +2270,6 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B28:D28"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2283,12 +2287,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="81" t="s">
+      <c r="A1" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="73"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="44"/>
     </row>
     <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="35" t="s">
@@ -2314,12 +2318,12 @@
       <c r="D4" s="41"/>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="80" t="s">
+      <c r="A6" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="77"/>
-      <c r="D6" s="73"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="44"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
@@ -2406,11 +2410,11 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="89" t="s">
+      <c r="A13" s="58" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="90"/>
-      <c r="C13" s="91"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="60"/>
       <c r="D13" s="20" t="str">
         <f>IF(D12="","", IF(SUM(D8:D11)&gt;0.8,"ĐẠT","CHƯA ĐẠT"))</f>
         <v/>
@@ -2418,12 +2422,12 @@
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="80" t="s">
+      <c r="A15" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="77"/>
-      <c r="C15" s="77"/>
-      <c r="D15" s="73"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="44"/>
     </row>
     <row r="16" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
@@ -2432,10 +2436,10 @@
       <c r="B16" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="79" t="s">
+      <c r="C16" s="45" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="73"/>
+      <c r="D16" s="44"/>
     </row>
     <row r="17" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="27" t="s">
@@ -2444,8 +2448,8 @@
       <c r="B17" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="84"/>
-      <c r="D17" s="85"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="54"/>
     </row>
     <row r="18" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="27" t="s">
@@ -2454,8 +2458,8 @@
       <c r="B18" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="84"/>
-      <c r="D18" s="85"/>
+      <c r="C18" s="53"/>
+      <c r="D18" s="54"/>
     </row>
     <row r="19" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="27" t="s">
@@ -2464,22 +2468,22 @@
       <c r="B19" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="84"/>
-      <c r="D19" s="85"/>
+      <c r="C19" s="53"/>
+      <c r="D19" s="54"/>
     </row>
     <row r="20" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="86" t="s">
+      <c r="A20" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="73"/>
-      <c r="C20" s="78" t="str">
+      <c r="B20" s="44"/>
+      <c r="C20" s="43" t="str">
         <f>IF(COUNTA(C17:C19)=0,"",
  IFERROR(VLOOKUP(C17,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B64
 +IFERROR(VLOOKUP(C18,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B65
 +IFERROR(VLOOKUP(C19,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B66)</f>
         <v/>
       </c>
-      <c r="D20" s="73"/>
+      <c r="D20" s="44"/>
     </row>
     <row r="21" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="33"/>
@@ -2488,96 +2492,100 @@
       <c r="D21" s="34"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="75" t="s">
+      <c r="A22" s="63" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
     </row>
     <row r="23" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="83" t="s">
+      <c r="A23" s="52" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="73"/>
-      <c r="C23" s="78" t="str">
+      <c r="B23" s="44"/>
+      <c r="C23" s="43" t="str">
         <f>IF(OR(D12="",C20=""),"",D12*'CẤU TRÚC &amp; TRỌNG SỐ'!B60+C20*'CẤU TRÚC &amp; TRỌNG SỐ'!B61)</f>
         <v/>
       </c>
-      <c r="D23" s="73"/>
+      <c r="D23" s="44"/>
     </row>
     <row r="24" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="72" t="s">
+      <c r="A24" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="B24" s="73"/>
-      <c r="C24" s="74" t="str">
+      <c r="B24" s="44"/>
+      <c r="C24" s="62" t="str">
         <f>IF(C23="","KHÔNG CÓ",
    IF(ROUND(C23,2)&lt;1,"CHƯA ĐẠT",
-      IF(AND(ROUND(C23,2)&gt;=1,ROUND(C23,2)&lt;1.2),"ĐẠT","TỐT")
+      IF(ROUND(C23,2)=1,"ĐẠT","TỐT")
    )
 )</f>
         <v>KHÔNG CÓ</v>
       </c>
-      <c r="D24" s="73"/>
+      <c r="D24" s="44"/>
     </row>
     <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="82"/>
-      <c r="B25" s="60"/>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
+      <c r="A25" s="50"/>
+      <c r="B25" s="51"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="51"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="87" t="s">
+      <c r="A26" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="77"/>
-      <c r="C26" s="77"/>
-      <c r="D26" s="73"/>
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="44"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="88" t="s">
+      <c r="B27" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="C27" s="77"/>
-      <c r="D27" s="73"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="44"/>
     </row>
     <row r="28" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B28" s="76" t="s">
+      <c r="B28" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="C28" s="77"/>
-      <c r="D28" s="73"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="44"/>
     </row>
     <row r="29" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B29" s="76" t="s">
+      <c r="B29" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="77"/>
-      <c r="D29" s="73"/>
+      <c r="C29" s="47"/>
+      <c r="D29" s="44"/>
     </row>
     <row r="30" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="B30" s="76" t="s">
+      <c r="B30" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="C30" s="77"/>
-      <c r="D30" s="73"/>
+      <c r="C30" s="47"/>
+      <c r="D30" s="44"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="xMEO7oWHm2o0A/zKZ1cbZgoj60M416AMIEEwH1xNc1SxnPRcpTDXwZzQGuI18O42T1maBUpoBnDujrn6JlYV8w==" saltValue="4TBryEnerdQHtfNbNwOYYQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="21">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="A15:D15"/>
@@ -2594,11 +2602,6 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:C11">
     <cfRule type="cellIs" dxfId="13" priority="4" operator="equal">
@@ -2679,25 +2682,25 @@
       <c r="A1" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
     </row>
     <row r="2" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="96" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A4" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
     </row>
     <row r="5" spans="1:4" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -2773,9 +2776,9 @@
       <c r="A11" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="64"/>
     </row>
     <row r="12" spans="1:4" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -2851,9 +2854,9 @@
       <c r="A18" s="93" t="s">
         <v>129</v>
       </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="44"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="64"/>
     </row>
     <row r="19" spans="1:5" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
@@ -3040,7 +3043,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8D0C41-9673-45B2-9EAD-BA190E719E0D}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.77734375" customWidth="1"/>
@@ -3095,6 +3098,14 @@
         <v>36</v>
       </c>
     </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="99" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" s="41" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -3104,7 +3115,7 @@
           <x14:formula1>
             <xm:f>'CẤU TRÚC &amp; TRỌNG SỐ'!$A$39:$A$42</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B6</xm:sqref>
+          <xm:sqref>B2:B7</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3132,25 +3143,25 @@
       <c r="A1" s="98" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="97" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
     </row>
     <row r="5" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">

</xml_diff>